<commit_message>
Anomalies SF1-MPS4 — 25/09/2026
</commit_message>
<xml_diff>
--- a/presentation/SF1-MPS4/anomalies.xlsx
+++ b/presentation/SF1-MPS4/anomalies.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1267,29 +1267,29 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>10368647</v>
+        <v>13667557</v>
       </c>
       <c r="B10" t="n">
-        <v>4204065</v>
+        <v>4002751599</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Remise en état la vanne eau de mer</t>
+          <t>INSPECTION GENERAL BRULEUR</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>OR000004204065</t>
+          <t>OR004002751599</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04-SECEMR</t>
+          <t>SF01-PS-PS04-SECGAZ-0F8301</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SECTION EAU DE MER DE L'ATELIER PS 4</t>
+          <t>BRULEUR A SOUFRE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1322,59 +1322,59 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P10" s="2" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>45715</v>
+        <v>46278</v>
       </c>
       <c r="R10" t="n">
         <v>1</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10368649</v>
+        <v>13667572</v>
       </c>
       <c r="B11" t="n">
-        <v>4204108</v>
+        <v>4002751693</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Etanchement fuite d'acide sur IAT</t>
+          <t>INSPECTION GENERALE DE POMPE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OR000004204108</t>
+          <t>OR004002751693</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04-SECACI-0E8304</t>
+          <t>SF01-PS-PS04-SECEAU-P8312B</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>REFROIDISSEUR ABSORPTION INTERMEDIAIRE</t>
+          <t>MOTOPOMP CIRCULAT B IN BALON VAPEUR HRS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1407,59 +1407,59 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P11" s="2" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>45715</v>
+        <v>46278</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10368692</v>
+        <v>13667574</v>
       </c>
       <c r="B12" t="n">
-        <v>4204142</v>
+        <v>4002751695</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ouverture et fermeture PV F/E/M</t>
+          <t>OMS RELEVE VIBRATION P8312B</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>OR000004204142</t>
+          <t>OR004002751695</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04-SECEMR</t>
+          <t>SF01-PS-PS04-SECEAU-P8312B</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SECTION EAU DE MER DE L'ATELIER PS 4</t>
+          <t>MOTOPOMP CIRCULAT B IN BALON VAPEUR HRS</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1492,59 +1492,59 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P12" s="2" t="n">
-        <v>46289</v>
+        <v>46292</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>45715</v>
+        <v>46278</v>
       </c>
       <c r="R12" t="n">
         <v>1</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>10148826</v>
+        <v>13667593</v>
       </c>
       <c r="B13" t="n">
-        <v>4206573</v>
+        <v>4002751728</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Installation monorail PV FA cooler</t>
+          <t>INSPECTION GENERALE DE POMPE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>OR000004206573</t>
+          <t>OR004002751728</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04-SECACI-0E8306</t>
+          <t>SF01-PS-PS04-SECACI-P8316A</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>REFROIDISSEUR ABSORPTION FINALE</t>
+          <t>MOTOPOMP VIDANGE P8316A ABSORP FINAL</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1577,59 +1577,59 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P13" s="2" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>45716</v>
+        <v>46278</v>
       </c>
       <c r="R13" t="n">
         <v>1</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>10368962</v>
+        <v>13667595</v>
       </c>
       <c r="B14" t="n">
-        <v>4212561</v>
+        <v>4002751730</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Démontage et remontage de la pompe 8304</t>
+          <t>OMS RELEVE VIBRATION P8316A</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>OR000004212561</t>
+          <t>OR004002751730</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04-SECACI-0P8304</t>
+          <t>SF01-PS-PS04-SECACI-P8316A</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MOTOPOMP ACIDE PRODUIT P8304</t>
+          <t>MOTOPOMP VIDANGE P8316A ABSORP FINAL</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1662,57 +1662,59 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P14" s="2" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>45720</v>
+        <v>46278</v>
       </c>
       <c r="R14" t="n">
         <v>1</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="n">
+        <v>13667596</v>
+      </c>
       <c r="B15" t="n">
-        <v>4298930</v>
+        <v>4002751731</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Montage vanne sur circuit de rinçage de</t>
+          <t>INSPECTION GENERALE DE POMPE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>OR000004298930</t>
+          <t>OR004002751731</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04-SECAIR-0C8301</t>
+          <t>SF01-PS-PS04-SECACI-P8316B</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TOUR DE SECHAGE C8301</t>
+          <t>MOTOPOMP VIDANGE P8316B ABSORP FINALE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1735,7 +1737,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1745,57 +1747,59 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P15" s="2" t="n">
-        <v>45836</v>
+        <v>46292</v>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>45744</v>
+        <v>46278</v>
       </c>
       <c r="R15" t="n">
         <v>1</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="n">
+        <v>13667598</v>
+      </c>
       <c r="B16" t="n">
-        <v>4302150</v>
+        <v>4002751733</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Préparation d'un collecteur de purge</t>
+          <t>OMS RELEVE VIBRATION P8316B</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>OR000004302150</t>
+          <t>OR004002751733</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04-SECSSL</t>
+          <t>SF01-PS-PS04-SECACI-P8316B</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>STOCKAGE SOUFRE LIQUIDE ATELIER PS 4</t>
+          <t>MOTOPOMP VIDANGE P8316B ABSORP FINALE</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1818,7 +1822,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1828,66 +1832,64 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P16" s="2" t="n">
-        <v>45836</v>
+        <v>46292</v>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>45745</v>
+        <v>46278</v>
       </c>
       <c r="R16" t="n">
         <v>1</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="n">
+        <v>13667632</v>
+      </c>
       <c r="B17" t="n">
-        <v>4002850076</v>
+        <v>4002751737</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Changement purgeur automatique coté four</t>
+          <t>INSPECTION GENERALE DE POMPE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>OR004002850076</t>
+          <t>OR004002751737</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04</t>
+          <t>SF01-PS-PS04-SECACI-0P8301</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ATELIER SULFURIQUE PS4</t>
+          <t>MOTOPOMP ACIDE P8301 SYSTÈME DE SECHAGE</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>SA-PC-PS4</t>
-        </is>
-      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>SF1-MPS4</t>
@@ -1905,7 +1907,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1915,66 +1917,64 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P17" s="2" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>46290</v>
+        <v>46278</v>
       </c>
       <c r="R17" t="n">
         <v>1</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="n">
+        <v>13667633</v>
+      </c>
       <c r="B18" t="n">
-        <v>4002850192</v>
+        <v>4002751738</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Etanchement fuite vapeur au niveau de ra</t>
+          <t>OMS RELEVE VIBRATION P8301</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>OR004002850192</t>
+          <t>OR004002751738</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04</t>
+          <t>SF01-PS-PS04-SECACI-0P8301</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ATELIER SULFURIQUE PS4</t>
+          <t>MOTOPOMP ACIDE P8301 SYSTÈME DE SECHAGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>SA-PC-PS4</t>
-        </is>
-      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>SF1-MPS4</t>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2002,66 +2002,64 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P18" s="2" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>46290</v>
+        <v>46278</v>
       </c>
       <c r="R18" t="n">
         <v>1</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>OT_COR_EGAL</t>
+          <t>OT exécution &lt;1 mois</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Agent de Saisie</t>
+          <t>Chef d'Atelier</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="n">
+        <v>13667602</v>
+      </c>
       <c r="B19" t="n">
-        <v>4002850199</v>
+        <v>4002751743</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Récupération circuit d'air de la turbine</t>
+          <t>INSPEC GENERAL TURBOSOUFFLANTE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>OR004002850199</t>
+          <t>OR004002751743</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SF01-PS-PS04</t>
+          <t>SF01-PS-PS04-SECAIR-0K8301</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>ATELIER SULFURIQUE PS4</t>
+          <t>SOUFFLANTE PRINCIPALE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>SA-PC-PS4</t>
-        </is>
-      </c>
+      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
           <t>SF1-MPS4</t>
@@ -2079,7 +2077,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2089,29 +2087,4111 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>MATAR1</t>
+          <t>IP1020260913</t>
         </is>
       </c>
       <c r="P19" s="2" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>46290</v>
+        <v>46278</v>
       </c>
       <c r="R19" t="n">
         <v>1</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>13667607</v>
+      </c>
+      <c r="B20" t="n">
+        <v>4002751748</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION K8301</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>OR004002751748</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECAIR-0K8301</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>SOUFFLANTE PRINCIPALE</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>13667615</v>
+      </c>
+      <c r="B21" t="n">
+        <v>4002751755</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERAL VENTILATEUR</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>OR004002751755</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECAIR-0K8302</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>VENTILATEUR PRIMAIRE</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>13667614</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4002751756</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>OR004002751756</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8305A</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>MOTOPOMP D'ALIMENTATION CHAUDIERE A</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q22" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>13667616</v>
+      </c>
+      <c r="B23" t="n">
+        <v>4002751757</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>OR004002751757</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8314A</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>MOTOPOMP RESERVOIR VIDANGE A HRS SYSTEM</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>13667618</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4002751759</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8314A</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>OR004002751759</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8314A</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>MOTOPOMP RESERVOIR VIDANGE A HRS SYSTEM</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R24" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>13667619</v>
+      </c>
+      <c r="B25" t="n">
+        <v>4002751760</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION K8302</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>OR004002751760</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECAIR-0K8302</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>VENTILATEUR PRIMAIRE</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R25" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>13667620</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4002751761</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8305A</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>OR004002751761</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8305A</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>MOTOPOMP D'ALIMENTATION CHAUDIERE A</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R26" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>13667624</v>
+      </c>
+      <c r="B27" t="n">
+        <v>4002751765</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>OR004002751765</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8314B</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>MOTOPOMP RESERVOIR VIDANGE B HRS SYSTEM</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R27" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>13667627</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4002751768</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>OR004002751768</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8305B</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>MOTOPOMP D'ALIMENTATION CHAUDIERE B</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>13667629</v>
+      </c>
+      <c r="B29" t="n">
+        <v>4002751770</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8314B</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>OR004002751770</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8314B</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>MOTOPOMP RESERVOIR VIDANGE B HRS SYSTEM</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R29" t="n">
+        <v>1</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>13667641</v>
+      </c>
+      <c r="B30" t="n">
+        <v>4002751772</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8305B</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>OR004002751772</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8305B</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>MOTOPOMP D'ALIMENTATION CHAUDIERE B</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R30" t="n">
+        <v>1</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>13667643</v>
+      </c>
+      <c r="B31" t="n">
+        <v>4002751774</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>INSPEC GENERAL TURBINE VAPEUR</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>OR004002751774</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECAIR-KT8301</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>TURBINE A VAPEUR</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R31" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>13667646</v>
+      </c>
+      <c r="B32" t="n">
+        <v>4002751777</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION KT8301</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>OR004002751777</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECAIR-KT8301</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>TURBINE A VAPEUR</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R32" t="n">
+        <v>1</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>13667636</v>
+      </c>
+      <c r="B33" t="n">
+        <v>4002751781</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>OR004002751781</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECACI-0P8302</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>MOTOPOMP ACIDE ABSORPTION INTERMEDIAIRE</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R33" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>13667638</v>
+      </c>
+      <c r="B34" t="n">
+        <v>4002751782</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8302</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>OR004002751782</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECACI-0P8302</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>MOTOPOMP ACIDE ABSORPTION INTERMEDIAIRE</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>13667660</v>
+      </c>
+      <c r="B35" t="n">
+        <v>4002751785</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>OR004002751785</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECACI-0P8303</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>MOTOPOMP ACIDE P8303 ABSORPTION FINALE</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R35" t="n">
+        <v>1</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>13667661</v>
+      </c>
+      <c r="B36" t="n">
+        <v>4002751786</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8303</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>OR004002751786</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECACI-0P8303</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>MOTOPOMP ACIDE P8303 ABSORPTION FINALE</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q36" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R36" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>13667662</v>
+      </c>
+      <c r="B37" t="n">
+        <v>4002751787</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>OR004002751787</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECACI-0P8304</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>MOTOPOMP ACIDE PRODUIT P8304</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R37" t="n">
+        <v>1</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>13667663</v>
+      </c>
+      <c r="B38" t="n">
+        <v>4002751788</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8304</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>OR004002751788</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECACI-0P8304</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>MOTOPOMP ACIDE PRODUIT P8304</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q38" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R38" t="n">
+        <v>1</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>13667667</v>
+      </c>
+      <c r="B39" t="n">
+        <v>4002751792</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>OR004002751792</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECSSL-P8201A</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>MOTOPOMPE SOUFRE P8201A AU FOUSSE SOUFRE</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R39" t="n">
+        <v>1</v>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>13667668</v>
+      </c>
+      <c r="B40" t="n">
+        <v>4002751793</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8201A</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>OR004002751793</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECSSL-P8201A</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>MOTOPOMPE SOUFRE P8201A AU FOUSSE SOUFRE</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q40" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R40" t="n">
+        <v>1</v>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>13667669</v>
+      </c>
+      <c r="B41" t="n">
+        <v>4002751794</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>OR004002751794</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECSSL-P8201B</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>MOTOPOMPE SOUFRE P8201B AU FOUSSE SOUFRE</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R41" t="n">
+        <v>1</v>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>13667710</v>
+      </c>
+      <c r="B42" t="n">
+        <v>4002751795</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8201B</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>OR004002751795</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECSSL-P8201B</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>MOTOPOMPE SOUFRE P8201B AU FOUSSE SOUFRE</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R42" t="n">
+        <v>1</v>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>13667558</v>
+      </c>
+      <c r="B43" t="n">
+        <v>4002751820</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION F8301</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>OR004002751820</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECGAZ-0F8301</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>BRULEUR A SOUFRE</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q43" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R43" t="n">
+        <v>1</v>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>13667559</v>
+      </c>
+      <c r="B44" t="n">
+        <v>4002751821</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>VERIFICATION POT DE GRAISSAGE</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>OR004002751821</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECGAZ-0F8301</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>BRULEUR A SOUFRE</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q44" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R44" t="n">
+        <v>1</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>13667680</v>
+      </c>
+      <c r="B45" t="n">
+        <v>4002751822</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERAL F8302</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>OR004002751822</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECGAZ-0F8302</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>FOUR A COMBUSTION F8302</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q45" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R45" t="n">
+        <v>1</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>13667701</v>
+      </c>
+      <c r="B46" t="n">
+        <v>4002751852</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>OR004002751852</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8309A</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>MOTOPOMP VIDANGE P8309A RESERVOIR</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q46" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R46" t="n">
+        <v>1</v>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>13667702</v>
+      </c>
+      <c r="B47" t="n">
+        <v>4002751853</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8309A</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>OR004002751853</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8309A</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>MOTOPOMP VIDANGE P8309A RESERVOIR</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q47" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R47" t="n">
+        <v>1</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>13667705</v>
+      </c>
+      <c r="B48" t="n">
+        <v>4002751856</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>OR004002751856</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8309B</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>MOTOPOMP VIDANG P8309B RESERVOIR VIDANG</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q48" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R48" t="n">
+        <v>1</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>13667706</v>
+      </c>
+      <c r="B49" t="n">
+        <v>4002751857</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8309B</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>OR004002751857</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8309B</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>MOTOPOMP VIDANG P8309B RESERVOIR VIDANG</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R49" t="n">
+        <v>1</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>13667709</v>
+      </c>
+      <c r="B50" t="n">
+        <v>4002751860</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>OR004002751860</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8311A</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>MOTOPOMP HEROS EAU ALIMENT CHAUDIERE A</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q50" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R50" t="n">
+        <v>1</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>13667720</v>
+      </c>
+      <c r="B51" t="n">
+        <v>4002751861</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>OR004002751861</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-0P8306</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>MOTOPOMP URGENCE ALIMENTATION CHAUDIERE</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R51" t="n">
+        <v>1</v>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>13667721</v>
+      </c>
+      <c r="B52" t="n">
+        <v>4002751862</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8311A</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>OR004002751862</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8311A</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>MOTOPOMP HEROS EAU ALIMENT CHAUDIERE A</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q52" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R52" t="n">
+        <v>1</v>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>13667723</v>
+      </c>
+      <c r="B53" t="n">
+        <v>4002751864</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8306</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>OR004002751864</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-0P8306</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>MOTOPOMP URGENCE ALIMENTATION CHAUDIERE</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q53" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R53" t="n">
+        <v>1</v>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>13667726</v>
+      </c>
+      <c r="B54" t="n">
+        <v>4002751867</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>OR004002751867</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8311B</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>MOTOPOMP HEROS EAU ALIMENT CHAUDIERE B</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q54" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R54" t="n">
+        <v>1</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>13667729</v>
+      </c>
+      <c r="B55" t="n">
+        <v>4002751870</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8311B</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>OR004002751870</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8311B</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>MOTOPOMP HEROS EAU ALIMENT CHAUDIERE B</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R55" t="n">
+        <v>1</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>13667733</v>
+      </c>
+      <c r="B56" t="n">
+        <v>4002751874</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>INSPECTION GENERALE DE POMPE</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>OR004002751874</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8312A</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>MOTOPOMP CIRCULAT A IN BALON VAPEUR HRS</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R56" t="n">
+        <v>1</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>13667737</v>
+      </c>
+      <c r="B57" t="n">
+        <v>4002751878</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>OMS RELEVE VIBRATION P8312A</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>OR004002751878</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEAU-P8312A</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>MOTOPOMP CIRCULAT A IN BALON VAPEUR HRS</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>LANC CCRP PART RIMP TEC  TàLT</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>IP1020260913</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q57" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="R57" t="n">
+        <v>1</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>OT exécution &lt;1 mois</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Chef d'Atelier</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Exécuter les ordres lancés conformément au planning hebdomadaire validé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>10368647</v>
+      </c>
+      <c r="B58" t="n">
+        <v>4204065</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Remise en état la vanne eau de mer</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>OR000004204065</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEMR</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>SECTION EAU DE MER DE L'ATELIER PS 4</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="Q58" s="2" t="n">
+        <v>45715</v>
+      </c>
+      <c r="R58" t="n">
+        <v>1</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
           <t>OT_COR_EGAL</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="T58" t="inlineStr">
         <is>
           <t>Agent de Saisie</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>10368649</v>
+      </c>
+      <c r="B59" t="n">
+        <v>4204108</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Etanchement fuite d'acide sur IAT</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>OR000004204108</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECACI-0E8304</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>REFROIDISSEUR ABSORPTION INTERMEDIAIRE</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="Q59" s="2" t="n">
+        <v>45715</v>
+      </c>
+      <c r="R59" t="n">
+        <v>1</v>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>10368692</v>
+      </c>
+      <c r="B60" t="n">
+        <v>4204142</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Ouverture et fermeture PV F/E/M</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>OR000004204142</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECEMR</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>SECTION EAU DE MER DE L'ATELIER PS 4</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="Q60" s="2" t="n">
+        <v>45715</v>
+      </c>
+      <c r="R60" t="n">
+        <v>1</v>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>10148826</v>
+      </c>
+      <c r="B61" t="n">
+        <v>4206573</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Installation monorail PV FA cooler</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>OR000004206573</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECACI-0E8306</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>REFROIDISSEUR ABSORPTION FINALE</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="Q61" s="2" t="n">
+        <v>45716</v>
+      </c>
+      <c r="R61" t="n">
+        <v>1</v>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>10368962</v>
+      </c>
+      <c r="B62" t="n">
+        <v>4212561</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Démontage et remontage de la pompe 8304</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>OR000004212561</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECACI-0P8304</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>MOTOPOMP ACIDE PRODUIT P8304</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="Q62" s="2" t="n">
+        <v>45720</v>
+      </c>
+      <c r="R62" t="n">
+        <v>1</v>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="n">
+        <v>4298930</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Montage vanne sur circuit de rinçage de</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>OR000004298930</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECAIR-0C8301</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TOUR DE SECHAGE C8301</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="n">
+        <v>45836</v>
+      </c>
+      <c r="Q63" s="2" t="n">
+        <v>45744</v>
+      </c>
+      <c r="R63" t="n">
+        <v>1</v>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="n">
+        <v>4302150</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Préparation d'un collecteur de purge</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>OR000004302150</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04-SECSSL</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>STOCKAGE SOUFRE LIQUIDE ATELIER PS 4</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="n">
+        <v>45836</v>
+      </c>
+      <c r="Q64" s="2" t="n">
+        <v>45745</v>
+      </c>
+      <c r="R64" t="n">
+        <v>1</v>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="n">
+        <v>4002850076</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Changement purgeur automatique coté four</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>OR004002850076</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>ATELIER SULFURIQUE PS4</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>SA-PC-PS4</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="Q65" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="R65" t="n">
+        <v>1</v>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="n">
+        <v>4002850192</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Etanchement fuite vapeur au niveau de ra</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>OR004002850192</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>ATELIER SULFURIQUE PS4</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>SA-PC-PS4</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="Q66" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="R66" t="n">
+        <v>1</v>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="n">
+        <v>4002850199</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Récupération circuit d'air de la turbine</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>OR004002850199</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>SF01-PS-PS04</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ATELIER SULFURIQUE PS4</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>SA-PC-PS4</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>SF1-MPS4</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>GM4</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>TCLO CONF CCRP JBFI PART RIMP</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>SOPL</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>MATAR1</t>
+        </is>
+      </c>
+      <c r="P67" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="Q67" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="R67" t="n">
+        <v>1</v>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>OT_COR_EGAL</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Agent de Saisie</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
         <is>
           <t>Contrôler la cohérence entre coûts budgétés et coûts réels, et corriger les OT dont les coûts ne sont pas cohérents (coûts réels = 0 ou égaux au budget).</t>
         </is>

</xml_diff>